<commit_message>
Estado de fecha, telefonos, redes y contacto ampliado
</commit_message>
<xml_diff>
--- a/data/festivales.xlsx
+++ b/data/festivales.xlsx
@@ -1146,7 +1146,11 @@
           <t>Francisco Nixon, Jonston</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bis.org/am_office/contact.htm</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1526,7 +1530,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>https://acandeloria.org/</t>
+          <t>https://blog.mundo-r.com/es/festivales-galicia/</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1588,7 @@
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>https://eternalmetal.cl/burgos-heavy-metal-2026-legion-dc/</t>
+          <t>https://metalhammer.es/burgos-heavy-metal-2026/</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2674,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>https://interestelarsevilla.com/</t>
+          <t>https://www.sevillaactualidad.com/cultura/593284-todo-lo-que-debes-saber-de-interestelar-sevilla-2026-artistas-horarios-y-desvios-en-las-lineas-de-autobuses/</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2736,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>https://metalkings.org/reports/10044</t>
+          <t>https://es.concerts-metal.com/concert_-_Metal_Strike_Fest_2026-242706.html</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3046,11 @@
           <t>Evaristo, El Drogas, Reincidentes</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>https://iberiafestival.com/contacto/</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3746,7 +3754,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>https://www.primaverasound.com/es/barcelona</t>
+          <t>https://www.primaverasound.com/es/barcelona/tickets-info-barcelona</t>
         </is>
       </c>
     </row>
@@ -4034,11 +4042,7 @@
           <t>Sexy Zebras, Carolina Durante, Ojete Calor, Siloé, Veintiuno, Brian de Calma, Depresión Sonora, El Nido, Fontán, Hoonine, Joe Crepúsculo, La Paloma</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>https://www.palenciasonora.com/cartel-palencia-sonora-2026/</t>
-        </is>
-      </c>
+      <c r="L64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4258,7 +4262,11 @@
           <t>La M.O.D.A., Barry B, La Habitación Roja, Carlos Ares, Rufus T. Firefly, BITA, Bauer, Bum Motion Club, Comandante Twin, Isaac Corrales, Marlena, Modelo</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>https://sentirbaeza.com/</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4354,11 +4362,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>https://antorchasfestival.com/</t>
-        </is>
-      </c>
+      <c r="L70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5408,11 +5412,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr"/>
       <c r="K89" s="2" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr">
-        <is>
-          <t>https://www.125.iberdrola.com/evento/iberdrola-music-festival-madrid/</t>
-        </is>
-      </c>
+      <c r="L89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6336,7 +6336,7 @@
       <c r="K106" s="2" t="inlineStr"/>
       <c r="L106" s="2" t="inlineStr">
         <is>
-          <t>https://piratafestival.com/es/</t>
+          <t>https://piratafestival.com/es/contacto/formulario</t>
         </is>
       </c>
     </row>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="L119" s="2" t="inlineStr">
         <is>
-          <t>https://bigsoundfestival.com/pontevedra/pontevedra</t>
+          <t>https://bigsoundfestival.com/contacto/?lang=es</t>
         </is>
       </c>
     </row>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="L128" s="2" t="inlineStr">
         <is>
-          <t>https://monegrosfestival.com/en</t>
+          <t>https://monegrosfestival.com/es</t>
         </is>
       </c>
     </row>
@@ -8480,7 +8480,7 @@
       </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>https://movidasound.com/ediciones-anteriores/edicion-2026/</t>
+          <t>https://movidasound.com/</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,11 @@
           <t>Ben Sims, DJ Pepo, Anika Kunst, DVS1, Elli Acula, Fleur Shore, Henrik Schwarz, Luca Agnelli, Prunk, Sam Divine</t>
         </is>
       </c>
-      <c r="L148" s="2" t="inlineStr"/>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.aquasella.shop/entradas</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -8776,11 +8780,7 @@
           <t>Love of Lesbian, La M.O.D.A., Siloé, Ultraligera, Carlos Ares, DJ Plan B, Fontán, Ginebras, KITAI, Karavana, Melifluo, Miss Caffeina</t>
         </is>
       </c>
-      <c r="L149" s="2" t="inlineStr">
-        <is>
-          <t>https://festivalmediterranea.com/726-2/</t>
-        </is>
-      </c>
+      <c r="L149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -9318,7 +9318,7 @@
       </c>
       <c r="L159" s="2" t="inlineStr">
         <is>
-          <t>https://festivalgigante.com/</t>
+          <t>https://festivalgigante.com/contacto/</t>
         </is>
       </c>
     </row>
@@ -11108,7 +11108,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17/10/2026 22:18</t>
+          <t>17/10/2026 22:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticketmaster: promotoras, entradas y 194 festivales
</commit_message>
<xml_diff>
--- a/data/festivales.xlsx
+++ b/data/festivales.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Festivales'!$A$1:$S$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Festivales'!$A$1:$S$195</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S191"/>
+  <dimension ref="A1:S195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -7457,7 +7457,11 @@
           <t>CANO, DAVS, JUNNIO</t>
         </is>
       </c>
-      <c r="K92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>Vida Festival</t>
+        </is>
+      </c>
       <c r="L92" s="2" t="inlineStr"/>
       <c r="M92" s="2" t="inlineStr">
         <is>
@@ -7466,7 +7470,11 @@
       </c>
       <c r="N92" s="3" t="inlineStr"/>
       <c r="O92" s="3" t="inlineStr"/>
-      <c r="P92" s="3" t="inlineStr"/>
+      <c r="P92" s="3" t="inlineStr">
+        <is>
+          <t>Sitback Produccions, S.L.</t>
+        </is>
+      </c>
       <c r="Q92" s="3" t="inlineStr"/>
       <c r="R92" s="3" t="inlineStr">
         <is>
@@ -14434,155 +14442,123 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Horteralia Cáceres 2026</t>
+          <t>Festa Presentació Vida Festival 2027: La Publicitat &amp; Bernal</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>Recinto Ferial de Cáceres</t>
+          <t>Antiga Fàbrica Estrella Damm</t>
         </is>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>Cáceres</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>Cáceres</t>
-        </is>
-      </c>
-      <c r="G185" s="3" t="inlineStr">
-        <is>
-          <t>Extremadura</t>
-        </is>
-      </c>
-      <c r="H185" s="2" t="inlineStr">
-        <is>
-          <t>Pop</t>
-        </is>
-      </c>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr"/>
+      <c r="H185" s="2" t="inlineStr"/>
       <c r="I185" s="4" t="inlineStr">
         <is>
-          <t>medio</t>
-        </is>
-      </c>
-      <c r="J185" s="2" t="inlineStr">
-        <is>
-          <t>CANO, CUPIDO, CYRIL KAMER</t>
-        </is>
-      </c>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr"/>
       <c r="K185" s="2" t="inlineStr">
         <is>
-          <t>Camela, Ladilla rusa, Amatria, Cherri Coke, El Gato con Jotas, Los Desgraciaus, Los Inhumanos, Nebulossa, Sharonne</t>
-        </is>
-      </c>
-      <c r="L185" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mevoyacaceres.com/festival-horteralia-de-caceres/</t>
-        </is>
-      </c>
+          <t>Vida Records &amp; Friends, Vida Festival</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr"/>
       <c r="M185" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N185" s="3" t="inlineStr">
-        <is>
-          <t>dpo@mediaprogramas.com</t>
-        </is>
-      </c>
+      <c r="N185" s="3" t="inlineStr"/>
       <c r="O185" s="3" t="inlineStr"/>
       <c r="P185" s="3" t="inlineStr">
         <is>
-          <t>En Mediaprogramas S.L</t>
-        </is>
-      </c>
-      <c r="Q185" s="3" t="inlineStr">
-        <is>
-          <t>informacion@ayto-caceres.es</t>
-        </is>
-      </c>
-      <c r="R185" s="3" t="inlineStr">
-        <is>
-          <t>618380445</t>
-        </is>
-      </c>
-      <c r="S185" s="3" t="inlineStr">
-        <is>
-          <t>https://www.ayto-caceres.es</t>
-        </is>
-      </c>
+          <t>Sitback Produccions, S.L.</t>
+        </is>
+      </c>
+      <c r="Q185" s="3" t="inlineStr"/>
+      <c r="R185" s="3" t="inlineStr"/>
+      <c r="S185" s="3" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Castañazo Rock 2026</t>
+          <t>Horteralia Cáceres 2026</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>Mercado ganadero</t>
+          <t>Recinto Ferial de Cáceres</t>
         </is>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>Chantada</t>
+          <t>Cáceres</t>
         </is>
       </c>
       <c r="F186" s="3" t="inlineStr">
         <is>
-          <t>Lugo</t>
+          <t>Cáceres</t>
         </is>
       </c>
       <c r="G186" s="3" t="inlineStr">
         <is>
-          <t>Galicia</t>
+          <t>Extremadura</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>Urbano, Pop, Rock, Punk</t>
+          <t>Pop</t>
         </is>
       </c>
       <c r="I186" s="4" t="inlineStr">
         <is>
-          <t>alto</t>
+          <t>medio</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr">
         <is>
-          <t>CUPIDO, JUNNIO, CANO</t>
+          <t>CANO, CUPIDO, CYRIL KAMER</t>
         </is>
       </c>
       <c r="K186" s="2" t="inlineStr">
         <is>
-          <t>Grande Amore, Kaotiko, Kumpania Algazarra, Moscow Death Brigade, Tremenda Jauría</t>
+          <t>Camela, Ladilla rusa, Amatria, Cherri Coke, El Gato con Jotas, Los Desgraciaus, Los Inhumanos, Nebulossa, Sharonne</t>
         </is>
       </c>
       <c r="L186" s="2" t="inlineStr">
         <is>
-          <t>https://castanhazo.com/venda-de-entradas/</t>
+          <t>https://www.mevoyacaceres.com/festival-horteralia-de-caceres/</t>
         </is>
       </c>
       <c r="M186" s="2" t="inlineStr">
@@ -14592,82 +14568,90 @@
       </c>
       <c r="N186" s="3" t="inlineStr">
         <is>
-          <t>attcliente@woutick.es</t>
+          <t>dpo@mediaprogramas.com</t>
         </is>
       </c>
       <c r="O186" s="3" t="inlineStr"/>
-      <c r="P186" s="3" t="inlineStr"/>
+      <c r="P186" s="3" t="inlineStr">
+        <is>
+          <t>En Mediaprogramas S.L</t>
+        </is>
+      </c>
       <c r="Q186" s="3" t="inlineStr">
         <is>
-          <t>concello@concellodechantada.es</t>
+          <t>informacion@ayto-caceres.es</t>
         </is>
       </c>
       <c r="R186" s="3" t="inlineStr">
         <is>
-          <t>614817558</t>
+          <t>618380445</t>
         </is>
       </c>
       <c r="S186" s="3" t="inlineStr">
         <is>
-          <t>https://www.concellodechantada.org</t>
+          <t>https://www.ayto-caceres.es</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Metal Bee 2026</t>
+          <t>Castañazo Rock 2026</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>Sala Matadero</t>
+          <t>Mercado ganadero</t>
         </is>
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>Ayora</t>
+          <t>Chantada</t>
         </is>
       </c>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Lugo</t>
         </is>
       </c>
       <c r="G187" s="3" t="inlineStr">
         <is>
-          <t>Comunidad Valenciana</t>
+          <t>Galicia</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Urbano, Pop, Rock, Punk</t>
         </is>
       </c>
       <c r="I187" s="4" t="inlineStr">
         <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J187" s="2" t="inlineStr"/>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>CUPIDO, JUNNIO, CANO</t>
+        </is>
+      </c>
       <c r="K187" s="2" t="inlineStr">
         <is>
-          <t>Leo Jiménez, Débler Eternia, Salduie, Seventh Hell, Six Burning Knives</t>
+          <t>Grande Amore, Kaotiko, Kumpania Algazarra, Moscow Death Brigade, Tremenda Jauría</t>
         </is>
       </c>
       <c r="L187" s="2" t="inlineStr">
         <is>
-          <t>http://tickets.salamatadero.com/es/matadero-live-music/iv-festival-metalbee/2026-11-28/</t>
+          <t>https://castanhazo.com/venda-de-entradas/</t>
         </is>
       </c>
       <c r="M187" s="2" t="inlineStr">
@@ -14677,71 +14661,71 @@
       </c>
       <c r="N187" s="3" t="inlineStr">
         <is>
-          <t>salamatadero@gmail.com</t>
+          <t>attcliente@woutick.es</t>
         </is>
       </c>
       <c r="O187" s="3" t="inlineStr"/>
       <c r="P187" s="3" t="inlineStr"/>
-      <c r="Q187" s="3" t="inlineStr"/>
-      <c r="R187" s="3" t="inlineStr"/>
+      <c r="Q187" s="3" t="inlineStr">
+        <is>
+          <t>concello@concellodechantada.es</t>
+        </is>
+      </c>
+      <c r="R187" s="3" t="inlineStr">
+        <is>
+          <t>614817558</t>
+        </is>
+      </c>
       <c r="S187" s="3" t="inlineStr">
         <is>
-          <t>https://www.ayora.es</t>
+          <t>https://www.concellodechantada.org</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Viña Rock 2027</t>
+          <t>GALILEO ROCK FEST</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>2027-04-29</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>Recinto Ferial de Villarrobledo</t>
+          <t>Sala Galileo Galilei</t>
         </is>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>Villarrobledo</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>Albacete</t>
-        </is>
-      </c>
-      <c r="G188" s="3" t="inlineStr">
-        <is>
-          <t>Castilla-La Mancha</t>
-        </is>
-      </c>
-      <c r="H188" s="2" t="inlineStr">
-        <is>
-          <t>Rock</t>
-        </is>
-      </c>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr"/>
+      <c r="H188" s="2" t="inlineStr"/>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t>medio</t>
-        </is>
-      </c>
-      <c r="J188" s="2" t="inlineStr">
-        <is>
-          <t>CUPIDO, JUNNIO</t>
-        </is>
-      </c>
-      <c r="K188" s="2" t="inlineStr"/>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr"/>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>Lion Rock Fest</t>
+        </is>
+      </c>
       <c r="L188" s="2" t="inlineStr"/>
       <c r="M188" s="2" t="inlineStr">
         <is>
@@ -14750,55 +14734,47 @@
       </c>
       <c r="N188" s="3" t="inlineStr"/>
       <c r="O188" s="3" t="inlineStr"/>
-      <c r="P188" s="3" t="inlineStr"/>
+      <c r="P188" s="3" t="inlineStr">
+        <is>
+          <t>Artisti-K Prod. Mus. y Cult, S.L.</t>
+        </is>
+      </c>
       <c r="Q188" s="3" t="inlineStr"/>
-      <c r="R188" s="3" t="inlineStr">
-        <is>
-          <t>736908127</t>
-        </is>
-      </c>
-      <c r="S188" s="3" t="inlineStr">
-        <is>
-          <t>https://villarrobledo.com</t>
-        </is>
-      </c>
+      <c r="R188" s="3" t="inlineStr"/>
+      <c r="S188" s="3" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>Interestelar Sevilla 2027</t>
+          <t>IBERDROLA MUSIC FESTIVAL VALENCIA - CONCIERTO ESTOPA</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>2027-05-14</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>Centro Andaluz de Arte Contemporáneo</t>
+          <t>Roig Arena</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
-      <c r="G189" s="3" t="inlineStr">
-        <is>
-          <t>Andalucía</t>
-        </is>
-      </c>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="G189" s="3" t="inlineStr"/>
       <c r="H189" s="2" t="inlineStr"/>
       <c r="I189" s="4" t="inlineStr">
         <is>
@@ -14806,140 +14782,156 @@
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr"/>
-      <c r="K189" s="2" t="inlineStr"/>
-      <c r="L189" s="2" t="inlineStr">
-        <is>
-          <t>https://conciertosensevilla.es/interestelar-sevilla-2027-viva-suecia-y-la-oreja-de-van-gogh-primeros-nombres-del-cartel/</t>
-        </is>
-      </c>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>IBERDROLA MUSIC FESTIVAL VALENCIA, Estopa</t>
+        </is>
+      </c>
+      <c r="L189" s="2" t="inlineStr"/>
       <c r="M189" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N189" s="3" t="inlineStr">
-        <is>
-          <t>hola@conciertosensevilla.es</t>
-        </is>
-      </c>
+      <c r="N189" s="3" t="inlineStr"/>
       <c r="O189" s="3" t="inlineStr"/>
-      <c r="P189" s="3" t="inlineStr"/>
+      <c r="P189" s="3" t="inlineStr">
+        <is>
+          <t>Live Nation España S.A.U.</t>
+        </is>
+      </c>
       <c r="Q189" s="3" t="inlineStr"/>
       <c r="R189" s="3" t="inlineStr"/>
-      <c r="S189" s="3" t="inlineStr">
-        <is>
-          <t>https://www.discoversevilla.city</t>
-        </is>
-      </c>
+      <c r="S189" s="3" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Primavera Sound Barcelona 2027</t>
+          <t>Metal Bee 2026</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>2027-06-03</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>2027-06-05</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>Parc del Fòrum</t>
+          <t>Sala Matadero</t>
         </is>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Ayora</t>
         </is>
       </c>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="G190" s="3" t="inlineStr">
         <is>
-          <t>Cataluña</t>
-        </is>
-      </c>
-      <c r="H190" s="2" t="inlineStr"/>
+          <t>Comunidad Valenciana</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>Metal</t>
+        </is>
+      </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
           <t>bajo</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr"/>
-      <c r="K190" s="2" t="inlineStr"/>
-      <c r="L190" s="2" t="inlineStr"/>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>Leo Jiménez, Débler Eternia, Salduie, Seventh Hell, Six Burning Knives</t>
+        </is>
+      </c>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>http://tickets.salamatadero.com/es/matadero-live-music/iv-festival-metalbee/2026-11-28/</t>
+        </is>
+      </c>
       <c r="M190" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N190" s="3" t="inlineStr"/>
+      <c r="N190" s="3" t="inlineStr">
+        <is>
+          <t>salamatadero@gmail.com</t>
+        </is>
+      </c>
       <c r="O190" s="3" t="inlineStr"/>
       <c r="P190" s="3" t="inlineStr"/>
       <c r="Q190" s="3" t="inlineStr"/>
-      <c r="R190" s="3" t="inlineStr">
-        <is>
-          <t>616401389</t>
-        </is>
-      </c>
+      <c r="R190" s="3" t="inlineStr"/>
       <c r="S190" s="3" t="inlineStr">
         <is>
-          <t>https://ajuntament.barcelona.cat</t>
+          <t>https://www.ayora.es</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Sónar 2027</t>
+          <t>Viña Rock 2027</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>2027-06-17</t>
+          <t>2027-04-29</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>2027-06-19</t>
+          <t>2027-05-01</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>Sónar de día - Fira Montjuïc</t>
+          <t>Recinto Ferial de Villarrobledo</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Villarrobledo</t>
         </is>
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Albacete</t>
         </is>
       </c>
       <c r="G191" s="3" t="inlineStr">
         <is>
-          <t>Cataluña</t>
-        </is>
-      </c>
-      <c r="H191" s="2" t="inlineStr"/>
+          <t>Castilla-La Mancha</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>Rock</t>
+        </is>
+      </c>
       <c r="I191" s="4" t="inlineStr">
         <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J191" s="2" t="inlineStr"/>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>CUPIDO, JUNNIO</t>
+        </is>
+      </c>
       <c r="K191" s="2" t="inlineStr"/>
       <c r="L191" s="2" t="inlineStr"/>
       <c r="M191" s="2" t="inlineStr">
@@ -14953,17 +14945,277 @@
       <c r="Q191" s="3" t="inlineStr"/>
       <c r="R191" s="3" t="inlineStr">
         <is>
+          <t>736908127</t>
+        </is>
+      </c>
+      <c r="S191" s="3" t="inlineStr">
+        <is>
+          <t>https://villarrobledo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Interestelar Sevilla 2027</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>2027-05-14</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>2027-05-15</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>Centro Andaluz de Arte Contemporáneo</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="G192" s="3" t="inlineStr">
+        <is>
+          <t>Andalucía</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr"/>
+      <c r="I192" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr"/>
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>https://conciertosensevilla.es/interestelar-sevilla-2027-viva-suecia-y-la-oreja-de-van-gogh-primeros-nombres-del-cartel/</t>
+        </is>
+      </c>
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N192" s="3" t="inlineStr">
+        <is>
+          <t>hola@conciertosensevilla.es</t>
+        </is>
+      </c>
+      <c r="O192" s="3" t="inlineStr"/>
+      <c r="P192" s="3" t="inlineStr"/>
+      <c r="Q192" s="3" t="inlineStr"/>
+      <c r="R192" s="3" t="inlineStr"/>
+      <c r="S192" s="3" t="inlineStr">
+        <is>
+          <t>https://www.discoversevilla.city</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>Primavera Sound Barcelona 2027</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-03</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-05</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>Parc del Fòrum</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="F193" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G193" s="3" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr"/>
+      <c r="I193" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr"/>
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="2" t="inlineStr"/>
+      <c r="M193" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N193" s="3" t="inlineStr"/>
+      <c r="O193" s="3" t="inlineStr"/>
+      <c r="P193" s="3" t="inlineStr"/>
+      <c r="Q193" s="3" t="inlineStr"/>
+      <c r="R193" s="3" t="inlineStr">
+        <is>
           <t>616401389</t>
         </is>
       </c>
-      <c r="S191" s="3" t="inlineStr">
+      <c r="S193" s="3" t="inlineStr">
         <is>
           <t>https://ajuntament.barcelona.cat</t>
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Sónar 2027</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-17</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-19</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Sónar de día - Fira Montjuïc</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G194" s="3" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr"/>
+      <c r="I194" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr"/>
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="2" t="inlineStr"/>
+      <c r="M194" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N194" s="3" t="inlineStr"/>
+      <c r="O194" s="3" t="inlineStr"/>
+      <c r="P194" s="3" t="inlineStr"/>
+      <c r="Q194" s="3" t="inlineStr"/>
+      <c r="R194" s="3" t="inlineStr">
+        <is>
+          <t>616401389</t>
+        </is>
+      </c>
+      <c r="S194" s="3" t="inlineStr">
+        <is>
+          <t>https://ajuntament.barcelona.cat</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>All Access Pass + Bus Super Early Bird - Circuit Festival 2027</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>2027-08-15</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>2027-08-15</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>Varios Recintos</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="F195" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G195" s="3" t="inlineStr"/>
+      <c r="H195" s="2" t="inlineStr"/>
+      <c r="I195" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr"/>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>Circuit Festival</t>
+        </is>
+      </c>
+      <c r="L195" s="2" t="inlineStr"/>
+      <c r="M195" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N195" s="3" t="inlineStr"/>
+      <c r="O195" s="3" t="inlineStr"/>
+      <c r="P195" s="3" t="inlineStr">
+        <is>
+          <t>Matinée 2000, SLU</t>
+        </is>
+      </c>
+      <c r="Q195" s="3" t="inlineStr"/>
+      <c r="R195" s="3" t="inlineStr"/>
+      <c r="S195" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S191"/>
+  <autoFilter ref="A1:S195"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14996,7 +15248,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>18/10/2026 08:02</t>
+          <t>18/10/2026 08:23</t>
         </is>
       </c>
     </row>
@@ -15007,7 +15259,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4">
@@ -15104,7 +15356,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -15124,7 +15376,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -15134,7 +15386,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Entradium integrado: organizador y precios
</commit_message>
<xml_diff>
--- a/data/festivales.xlsx
+++ b/data/festivales.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Festivales'!$A$1:$S$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Festivales'!$A$1:$S$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S195"/>
+  <dimension ref="A1:S200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -6063,7 +6063,11 @@
         </is>
       </c>
       <c r="O73" s="3" t="inlineStr"/>
-      <c r="P73" s="3" t="inlineStr"/>
+      <c r="P73" s="3" t="inlineStr">
+        <is>
+          <t>COPILOTS EVENTS, S.L.</t>
+        </is>
+      </c>
       <c r="Q73" s="3" t="inlineStr"/>
       <c r="R73" s="3" t="inlineStr">
         <is>
@@ -7235,7 +7239,11 @@
       </c>
       <c r="N89" s="3" t="inlineStr"/>
       <c r="O89" s="3" t="inlineStr"/>
-      <c r="P89" s="3" t="inlineStr"/>
+      <c r="P89" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THE RAVE KULTURE </t>
+        </is>
+      </c>
       <c r="Q89" s="3" t="inlineStr"/>
       <c r="R89" s="3" t="inlineStr"/>
       <c r="S89" s="3" t="inlineStr">
@@ -10672,7 +10680,11 @@
         </is>
       </c>
       <c r="O134" s="3" t="inlineStr"/>
-      <c r="P134" s="3" t="inlineStr"/>
+      <c r="P134" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLUB MUTANTE </t>
+        </is>
+      </c>
       <c r="Q134" s="3" t="inlineStr">
         <is>
           <t>ventanillaunica@borja.es</t>
@@ -13266,7 +13278,11 @@
       </c>
       <c r="N168" s="3" t="inlineStr"/>
       <c r="O168" s="3" t="inlineStr"/>
-      <c r="P168" s="3" t="inlineStr"/>
+      <c r="P168" s="3" t="inlineStr">
+        <is>
+          <t>Debeat Swing</t>
+        </is>
+      </c>
       <c r="Q168" s="3" t="inlineStr"/>
       <c r="R168" s="3" t="inlineStr"/>
       <c r="S168" s="3" t="inlineStr"/>
@@ -14596,182 +14612,174 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Castañazo Rock 2026</t>
+          <t>La CHICA FEST. Actuación de Elegante embustero. Formato trío</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>Mercado ganadero</t>
+          <t xml:space="preserve">Pub La chica de ayer </t>
         </is>
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>Chantada</t>
-        </is>
-      </c>
-      <c r="F187" s="3" t="inlineStr">
-        <is>
-          <t>Lugo</t>
-        </is>
-      </c>
-      <c r="G187" s="3" t="inlineStr">
-        <is>
-          <t>Galicia</t>
-        </is>
-      </c>
-      <c r="H187" s="2" t="inlineStr">
-        <is>
-          <t>Urbano, Pop, Rock, Punk</t>
-        </is>
-      </c>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="inlineStr"/>
+      <c r="G187" s="3" t="inlineStr"/>
+      <c r="H187" s="2" t="inlineStr"/>
       <c r="I187" s="4" t="inlineStr">
         <is>
-          <t>alto</t>
-        </is>
-      </c>
-      <c r="J187" s="2" t="inlineStr">
-        <is>
-          <t>CUPIDO, JUNNIO, CANO</t>
-        </is>
-      </c>
-      <c r="K187" s="2" t="inlineStr">
-        <is>
-          <t>Grande Amore, Kaotiko, Kumpania Algazarra, Moscow Death Brigade, Tremenda Jauría</t>
-        </is>
-      </c>
-      <c r="L187" s="2" t="inlineStr">
-        <is>
-          <t>https://castanhazo.com/venda-de-entradas/</t>
-        </is>
-      </c>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr"/>
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="2" t="inlineStr"/>
       <c r="M187" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N187" s="3" t="inlineStr">
-        <is>
-          <t>attcliente@woutick.es</t>
-        </is>
-      </c>
+      <c r="N187" s="3" t="inlineStr"/>
       <c r="O187" s="3" t="inlineStr"/>
-      <c r="P187" s="3" t="inlineStr"/>
-      <c r="Q187" s="3" t="inlineStr">
-        <is>
-          <t>concello@concellodechantada.es</t>
-        </is>
-      </c>
-      <c r="R187" s="3" t="inlineStr">
-        <is>
-          <t>614817558</t>
-        </is>
-      </c>
-      <c r="S187" s="3" t="inlineStr">
-        <is>
-          <t>https://www.concellodechantada.org</t>
-        </is>
-      </c>
+      <c r="P187" s="3" t="inlineStr">
+        <is>
+          <t>La chica Fest</t>
+        </is>
+      </c>
+      <c r="Q187" s="3" t="inlineStr"/>
+      <c r="R187" s="3" t="inlineStr"/>
+      <c r="S187" s="3" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>GALILEO ROCK FEST</t>
+          <t>Castañazo Rock 2026</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>Sala Galileo Galilei</t>
+          <t>Mercado ganadero</t>
         </is>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Chantada</t>
         </is>
       </c>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>Madrid</t>
-        </is>
-      </c>
-      <c r="G188" s="3" t="inlineStr"/>
-      <c r="H188" s="2" t="inlineStr"/>
+          <t>Lugo</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr">
+        <is>
+          <t>Galicia</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>Urbano, Pop, Rock, Punk</t>
+        </is>
+      </c>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J188" s="2" t="inlineStr"/>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>CUPIDO, JUNNIO, CANO</t>
+        </is>
+      </c>
       <c r="K188" s="2" t="inlineStr">
         <is>
-          <t>Lion Rock Fest</t>
-        </is>
-      </c>
-      <c r="L188" s="2" t="inlineStr"/>
+          <t>Grande Amore, Kaotiko, Kumpania Algazarra, Moscow Death Brigade, Tremenda Jauría</t>
+        </is>
+      </c>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>https://castanhazo.com/venda-de-entradas/</t>
+        </is>
+      </c>
       <c r="M188" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N188" s="3" t="inlineStr"/>
+      <c r="N188" s="3" t="inlineStr">
+        <is>
+          <t>attcliente@woutick.es</t>
+        </is>
+      </c>
       <c r="O188" s="3" t="inlineStr"/>
-      <c r="P188" s="3" t="inlineStr">
-        <is>
-          <t>Artisti-K Prod. Mus. y Cult, S.L.</t>
-        </is>
-      </c>
-      <c r="Q188" s="3" t="inlineStr"/>
-      <c r="R188" s="3" t="inlineStr"/>
-      <c r="S188" s="3" t="inlineStr"/>
+      <c r="P188" s="3" t="inlineStr"/>
+      <c r="Q188" s="3" t="inlineStr">
+        <is>
+          <t>concello@concellodechantada.es</t>
+        </is>
+      </c>
+      <c r="R188" s="3" t="inlineStr">
+        <is>
+          <t>614817558</t>
+        </is>
+      </c>
+      <c r="S188" s="3" t="inlineStr">
+        <is>
+          <t>https://www.concellodechantada.org</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>IBERDROLA MUSIC FESTIVAL VALENCIA - CONCIERTO ESTOPA</t>
+          <t>GALILEO ROCK FEST</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>Roig Arena</t>
+          <t>Sala Galileo Galilei</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr"/>
@@ -14784,7 +14792,7 @@
       <c r="J189" s="2" t="inlineStr"/>
       <c r="K189" s="2" t="inlineStr">
         <is>
-          <t>IBERDROLA MUSIC FESTIVAL VALENCIA, Estopa</t>
+          <t>Lion Rock Fest</t>
         </is>
       </c>
       <c r="L189" s="2" t="inlineStr"/>
@@ -14797,7 +14805,7 @@
       <c r="O189" s="3" t="inlineStr"/>
       <c r="P189" s="3" t="inlineStr">
         <is>
-          <t>Live Nation España S.A.U.</t>
+          <t>Artisti-K Prod. Mus. y Cult, S.L.</t>
         </is>
       </c>
       <c r="Q189" s="3" t="inlineStr"/>
@@ -14807,131 +14815,91 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Metal Bee 2026</t>
+          <t>ALFAJARÍN, CULTURA ELECTRÓNICA 2026 (The Raven Clan)</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>Sala Matadero</t>
+          <t xml:space="preserve">SALÓN CULTURAL “LA PORTAZA” </t>
         </is>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>Ayora</t>
-        </is>
-      </c>
-      <c r="F190" s="3" t="inlineStr">
-        <is>
-          <t>Valencia</t>
-        </is>
-      </c>
-      <c r="G190" s="3" t="inlineStr">
-        <is>
-          <t>Comunidad Valenciana</t>
-        </is>
-      </c>
-      <c r="H190" s="2" t="inlineStr">
-        <is>
-          <t>Metal</t>
-        </is>
-      </c>
+          <t>Alfajarín</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="inlineStr"/>
+      <c r="G190" s="3" t="inlineStr"/>
+      <c r="H190" s="2" t="inlineStr"/>
       <c r="I190" s="4" t="inlineStr">
         <is>
           <t>bajo</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr"/>
-      <c r="K190" s="2" t="inlineStr">
-        <is>
-          <t>Leo Jiménez, Débler Eternia, Salduie, Seventh Hell, Six Burning Knives</t>
-        </is>
-      </c>
-      <c r="L190" s="2" t="inlineStr">
-        <is>
-          <t>http://tickets.salamatadero.com/es/matadero-live-music/iv-festival-metalbee/2026-11-28/</t>
-        </is>
-      </c>
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="2" t="inlineStr"/>
       <c r="M190" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N190" s="3" t="inlineStr">
-        <is>
-          <t>salamatadero@gmail.com</t>
-        </is>
-      </c>
+      <c r="N190" s="3" t="inlineStr"/>
       <c r="O190" s="3" t="inlineStr"/>
-      <c r="P190" s="3" t="inlineStr"/>
+      <c r="P190" s="3" t="inlineStr">
+        <is>
+          <t>AYUNTAMIENTO DE ALFAJARÍN</t>
+        </is>
+      </c>
       <c r="Q190" s="3" t="inlineStr"/>
       <c r="R190" s="3" t="inlineStr"/>
-      <c r="S190" s="3" t="inlineStr">
-        <is>
-          <t>https://www.ayora.es</t>
-        </is>
-      </c>
+      <c r="S190" s="3" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Viña Rock 2027</t>
+          <t>IV FESTIVAL SEVILLA SIXTIES SOUND</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>2027-04-29</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>Recinto Ferial de Villarrobledo</t>
+          <t>SALA EVEN</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>Villarrobledo</t>
-        </is>
-      </c>
-      <c r="F191" s="3" t="inlineStr">
-        <is>
-          <t>Albacete</t>
-        </is>
-      </c>
-      <c r="G191" s="3" t="inlineStr">
-        <is>
-          <t>Castilla-La Mancha</t>
-        </is>
-      </c>
-      <c r="H191" s="2" t="inlineStr">
-        <is>
-          <t>Rock</t>
-        </is>
-      </c>
+          <t>SEVILLA</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr"/>
+      <c r="G191" s="3" t="inlineStr"/>
+      <c r="H191" s="2" t="inlineStr"/>
       <c r="I191" s="4" t="inlineStr">
         <is>
-          <t>medio</t>
-        </is>
-      </c>
-      <c r="J191" s="2" t="inlineStr">
-        <is>
-          <t>CUPIDO, JUNNIO</t>
-        </is>
-      </c>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr"/>
       <c r="K191" s="2" t="inlineStr"/>
       <c r="L191" s="2" t="inlineStr"/>
       <c r="M191" s="2" t="inlineStr">
@@ -14941,55 +14909,47 @@
       </c>
       <c r="N191" s="3" t="inlineStr"/>
       <c r="O191" s="3" t="inlineStr"/>
-      <c r="P191" s="3" t="inlineStr"/>
+      <c r="P191" s="3" t="inlineStr">
+        <is>
+          <t>SIXTIES SOUND SEVILLA</t>
+        </is>
+      </c>
       <c r="Q191" s="3" t="inlineStr"/>
-      <c r="R191" s="3" t="inlineStr">
-        <is>
-          <t>736908127</t>
-        </is>
-      </c>
-      <c r="S191" s="3" t="inlineStr">
-        <is>
-          <t>https://villarrobledo.com</t>
-        </is>
-      </c>
+      <c r="R191" s="3" t="inlineStr"/>
+      <c r="S191" s="3" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Interestelar Sevilla 2027</t>
+          <t>IBERDROLA MUSIC FESTIVAL VALENCIA - CONCIERTO ESTOPA</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>2027-05-14</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>Centro Andaluz de Arte Contemporáneo</t>
+          <t>Roig Arena</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="F192" s="3" t="inlineStr">
         <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
-      <c r="G192" s="3" t="inlineStr">
-        <is>
-          <t>Andalucía</t>
-        </is>
-      </c>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="G192" s="3" t="inlineStr"/>
       <c r="H192" s="2" t="inlineStr"/>
       <c r="I192" s="4" t="inlineStr">
         <is>
@@ -14997,133 +14957,133 @@
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr"/>
-      <c r="K192" s="2" t="inlineStr"/>
-      <c r="L192" s="2" t="inlineStr">
-        <is>
-          <t>https://conciertosensevilla.es/interestelar-sevilla-2027-viva-suecia-y-la-oreja-de-van-gogh-primeros-nombres-del-cartel/</t>
-        </is>
-      </c>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>IBERDROLA MUSIC FESTIVAL VALENCIA, Estopa</t>
+        </is>
+      </c>
+      <c r="L192" s="2" t="inlineStr"/>
       <c r="M192" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N192" s="3" t="inlineStr">
-        <is>
-          <t>hola@conciertosensevilla.es</t>
-        </is>
-      </c>
+      <c r="N192" s="3" t="inlineStr"/>
       <c r="O192" s="3" t="inlineStr"/>
-      <c r="P192" s="3" t="inlineStr"/>
+      <c r="P192" s="3" t="inlineStr">
+        <is>
+          <t>Live Nation España S.A.U.</t>
+        </is>
+      </c>
       <c r="Q192" s="3" t="inlineStr"/>
       <c r="R192" s="3" t="inlineStr"/>
-      <c r="S192" s="3" t="inlineStr">
-        <is>
-          <t>https://www.discoversevilla.city</t>
-        </is>
-      </c>
+      <c r="S192" s="3" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Primavera Sound Barcelona 2027</t>
+          <t>Metal Bee 2026</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>2027-06-03</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>2027-06-05</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>Parc del Fòrum</t>
+          <t>Sala Matadero</t>
         </is>
       </c>
       <c r="E193" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Ayora</t>
         </is>
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="G193" s="3" t="inlineStr">
         <is>
-          <t>Cataluña</t>
-        </is>
-      </c>
-      <c r="H193" s="2" t="inlineStr"/>
+          <t>Comunidad Valenciana</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>Metal</t>
+        </is>
+      </c>
       <c r="I193" s="4" t="inlineStr">
         <is>
           <t>bajo</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr"/>
-      <c r="K193" s="2" t="inlineStr"/>
-      <c r="L193" s="2" t="inlineStr"/>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>Leo Jiménez, Débler Eternia, Salduie, Seventh Hell, Six Burning Knives</t>
+        </is>
+      </c>
+      <c r="L193" s="2" t="inlineStr">
+        <is>
+          <t>http://tickets.salamatadero.com/es/matadero-live-music/iv-festival-metalbee/2026-11-28/</t>
+        </is>
+      </c>
       <c r="M193" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N193" s="3" t="inlineStr"/>
+      <c r="N193" s="3" t="inlineStr">
+        <is>
+          <t>salamatadero@gmail.com</t>
+        </is>
+      </c>
       <c r="O193" s="3" t="inlineStr"/>
       <c r="P193" s="3" t="inlineStr"/>
       <c r="Q193" s="3" t="inlineStr"/>
-      <c r="R193" s="3" t="inlineStr">
-        <is>
-          <t>616401389</t>
-        </is>
-      </c>
+      <c r="R193" s="3" t="inlineStr"/>
       <c r="S193" s="3" t="inlineStr">
         <is>
-          <t>https://ajuntament.barcelona.cat</t>
+          <t>https://www.ayora.es</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Sónar 2027</t>
+          <t>NoTeMofest acto 4</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>2027-06-17</t>
+          <t>2027-02-20</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>2027-06-19</t>
+          <t>2027-02-20</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>Sónar de día - Fira Montjuïc</t>
+          <t>Andén 56</t>
         </is>
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="F194" s="3" t="inlineStr">
-        <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="G194" s="3" t="inlineStr">
-        <is>
-          <t>Cataluña</t>
-        </is>
-      </c>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="inlineStr"/>
+      <c r="G194" s="3" t="inlineStr"/>
       <c r="H194" s="2" t="inlineStr"/>
       <c r="I194" s="4" t="inlineStr">
         <is>
@@ -15140,63 +15100,67 @@
       </c>
       <c r="N194" s="3" t="inlineStr"/>
       <c r="O194" s="3" t="inlineStr"/>
-      <c r="P194" s="3" t="inlineStr"/>
+      <c r="P194" s="3" t="inlineStr">
+        <is>
+          <t>Steel Souls Producciones</t>
+        </is>
+      </c>
       <c r="Q194" s="3" t="inlineStr"/>
-      <c r="R194" s="3" t="inlineStr">
-        <is>
-          <t>616401389</t>
-        </is>
-      </c>
-      <c r="S194" s="3" t="inlineStr">
-        <is>
-          <t>https://ajuntament.barcelona.cat</t>
-        </is>
-      </c>
+      <c r="R194" s="3" t="inlineStr"/>
+      <c r="S194" s="3" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>All Access Pass + Bus Super Early Bird - Circuit Festival 2027</t>
+          <t>Viña Rock 2027</t>
         </is>
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-04-29</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>2027-08-15</t>
+          <t>2027-05-01</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Varios Recintos</t>
+          <t>Recinto Ferial de Villarrobledo</t>
         </is>
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Villarrobledo</t>
         </is>
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="G195" s="3" t="inlineStr"/>
-      <c r="H195" s="2" t="inlineStr"/>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="G195" s="3" t="inlineStr">
+        <is>
+          <t>Castilla-La Mancha</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>Rock</t>
+        </is>
+      </c>
       <c r="I195" s="4" t="inlineStr">
         <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J195" s="2" t="inlineStr"/>
-      <c r="K195" s="2" t="inlineStr">
-        <is>
-          <t>Circuit Festival</t>
-        </is>
-      </c>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>CUPIDO, JUNNIO</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr"/>
       <c r="L195" s="2" t="inlineStr"/>
       <c r="M195" s="2" t="inlineStr">
         <is>
@@ -15205,17 +15169,334 @@
       </c>
       <c r="N195" s="3" t="inlineStr"/>
       <c r="O195" s="3" t="inlineStr"/>
-      <c r="P195" s="3" t="inlineStr">
+      <c r="P195" s="3" t="inlineStr"/>
+      <c r="Q195" s="3" t="inlineStr"/>
+      <c r="R195" s="3" t="inlineStr">
+        <is>
+          <t>736908127</t>
+        </is>
+      </c>
+      <c r="S195" s="3" t="inlineStr">
+        <is>
+          <t>https://villarrobledo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Interestelar Sevilla 2027</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>2027-05-14</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>2027-05-15</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Centro Andaluz de Arte Contemporáneo</t>
+        </is>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="F196" s="3" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="G196" s="3" t="inlineStr">
+        <is>
+          <t>Andalucía</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr"/>
+      <c r="I196" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr"/>
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="2" t="inlineStr">
+        <is>
+          <t>https://conciertosensevilla.es/interestelar-sevilla-2027-viva-suecia-y-la-oreja-de-van-gogh-primeros-nombres-del-cartel/</t>
+        </is>
+      </c>
+      <c r="M196" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N196" s="3" t="inlineStr">
+        <is>
+          <t>hola@conciertosensevilla.es</t>
+        </is>
+      </c>
+      <c r="O196" s="3" t="inlineStr"/>
+      <c r="P196" s="3" t="inlineStr"/>
+      <c r="Q196" s="3" t="inlineStr"/>
+      <c r="R196" s="3" t="inlineStr"/>
+      <c r="S196" s="3" t="inlineStr">
+        <is>
+          <t>https://www.discoversevilla.city</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>Primavera Sound Barcelona 2027</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-03</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-05</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>Parc del Fòrum</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G197" s="3" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr"/>
+      <c r="I197" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr"/>
+      <c r="K197" s="2" t="inlineStr"/>
+      <c r="L197" s="2" t="inlineStr"/>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N197" s="3" t="inlineStr"/>
+      <c r="O197" s="3" t="inlineStr"/>
+      <c r="P197" s="3" t="inlineStr"/>
+      <c r="Q197" s="3" t="inlineStr"/>
+      <c r="R197" s="3" t="inlineStr">
+        <is>
+          <t>616401389</t>
+        </is>
+      </c>
+      <c r="S197" s="3" t="inlineStr">
+        <is>
+          <t>https://ajuntament.barcelona.cat</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>Sónar 2027</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-17</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>2027-06-19</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>Sónar de día - Fira Montjuïc</t>
+        </is>
+      </c>
+      <c r="E198" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="F198" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G198" s="3" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr"/>
+      <c r="I198" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr"/>
+      <c r="K198" s="2" t="inlineStr"/>
+      <c r="L198" s="2" t="inlineStr"/>
+      <c r="M198" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N198" s="3" t="inlineStr"/>
+      <c r="O198" s="3" t="inlineStr"/>
+      <c r="P198" s="3" t="inlineStr"/>
+      <c r="Q198" s="3" t="inlineStr"/>
+      <c r="R198" s="3" t="inlineStr">
+        <is>
+          <t>616401389</t>
+        </is>
+      </c>
+      <c r="S198" s="3" t="inlineStr">
+        <is>
+          <t>https://ajuntament.barcelona.cat</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>All Access Pass + Bus Super Early Bird - Circuit Festival 2027</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>2027-08-15</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>2027-08-15</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>Varios Recintos</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G199" s="3" t="inlineStr"/>
+      <c r="H199" s="2" t="inlineStr"/>
+      <c r="I199" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr"/>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t>Circuit Festival</t>
+        </is>
+      </c>
+      <c r="L199" s="2" t="inlineStr"/>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N199" s="3" t="inlineStr"/>
+      <c r="O199" s="3" t="inlineStr"/>
+      <c r="P199" s="3" t="inlineStr">
         <is>
           <t>Matinée 2000, SLU</t>
         </is>
       </c>
-      <c r="Q195" s="3" t="inlineStr"/>
-      <c r="R195" s="3" t="inlineStr"/>
-      <c r="S195" s="3" t="inlineStr"/>
+      <c r="Q199" s="3" t="inlineStr"/>
+      <c r="R199" s="3" t="inlineStr"/>
+      <c r="S199" s="3" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Scanner bilbao</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>2027-09-17</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>2027-09-17</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>D8 sorkuntza</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>Bilbao</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="inlineStr"/>
+      <c r="G200" s="3" t="inlineStr"/>
+      <c r="H200" s="2" t="inlineStr"/>
+      <c r="I200" s="4" t="inlineStr">
+        <is>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr"/>
+      <c r="K200" s="2" t="inlineStr"/>
+      <c r="L200" s="2" t="inlineStr"/>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+      <c r="N200" s="3" t="inlineStr"/>
+      <c r="O200" s="3" t="inlineStr"/>
+      <c r="P200" s="3" t="inlineStr">
+        <is>
+          <t>Copilots Events</t>
+        </is>
+      </c>
+      <c r="Q200" s="3" t="inlineStr"/>
+      <c r="R200" s="3" t="inlineStr"/>
+      <c r="S200" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S195"/>
+  <autoFilter ref="A1:S200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15248,7 +15529,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>18/10/2026 08:23</t>
+          <t>18/10/2026 08:40</t>
         </is>
       </c>
     </row>
@@ -15259,7 +15540,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4">
@@ -15269,7 +15550,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
@@ -15296,7 +15577,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -15366,7 +15647,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
@@ -15376,7 +15657,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -15386,7 +15667,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Azul Rabat, filtro confirmados, limpieza de fichas
</commit_message>
<xml_diff>
--- a/data/festivales.xlsx
+++ b/data/festivales.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Festivales'!$A$1:$S$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Festivales'!$A$1:$S$198</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S200"/>
+  <dimension ref="A1:S198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -653,8 +653,16 @@
           <t>CRASH MUSIC S.L</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>ayto@aytoalmeria.es</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>626900000</t>
+        </is>
+      </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
           <t>http://sede.aytoalmeria.es</t>
@@ -1119,16 +1127,8 @@
       </c>
       <c r="O8" s="3" t="inlineStr"/>
       <c r="P8" s="3" t="inlineStr"/>
-      <c r="Q8" s="3" t="inlineStr">
-        <is>
-          <t>registro@ayora.es</t>
-        </is>
-      </c>
-      <c r="R8" s="3" t="inlineStr">
-        <is>
-          <t>880898509</t>
-        </is>
-      </c>
+      <c r="Q8" s="3" t="inlineStr"/>
+      <c r="R8" s="3" t="inlineStr"/>
       <c r="S8" s="3" t="inlineStr">
         <is>
           <t>https://www.ayora.es</t>
@@ -2035,8 +2035,16 @@
       </c>
       <c r="O20" s="3" t="inlineStr"/>
       <c r="P20" s="3" t="inlineStr"/>
-      <c r="Q20" s="3" t="inlineStr"/>
-      <c r="R20" s="3" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>servicio010@aytoburgos.es</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>623921931</t>
+        </is>
+      </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
           <t>https://www.aytoburgos.es</t>
@@ -2314,7 +2322,7 @@
       <c r="Q24" s="3" t="inlineStr"/>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>792324372</t>
+          <t>792317685</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
@@ -2707,7 +2715,7 @@
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
-          <t>644550455</t>
+          <t>647164776</t>
         </is>
       </c>
       <c r="S29" s="3" t="inlineStr">
@@ -4389,7 +4397,7 @@
       </c>
       <c r="R51" s="3" t="inlineStr">
         <is>
-          <t>722515367</t>
+          <t>600961018</t>
         </is>
       </c>
       <c r="S51" s="3" t="inlineStr">
@@ -4462,7 +4470,7 @@
       </c>
       <c r="R52" s="3" t="inlineStr">
         <is>
-          <t>686165275</t>
+          <t>800729525</t>
         </is>
       </c>
       <c r="S52" s="3" t="inlineStr">
@@ -4624,7 +4632,7 @@
       </c>
       <c r="R54" s="3" t="inlineStr">
         <is>
-          <t>644550455</t>
+          <t>647164776</t>
         </is>
       </c>
       <c r="S54" s="3" t="inlineStr">
@@ -5812,7 +5820,7 @@
       <c r="Q70" s="3" t="inlineStr"/>
       <c r="R70" s="3" t="inlineStr">
         <is>
-          <t>792324372</t>
+          <t>792317685</t>
         </is>
       </c>
       <c r="S70" s="3" t="inlineStr">
@@ -5897,7 +5905,7 @@
       </c>
       <c r="R71" s="3" t="inlineStr">
         <is>
-          <t>639444225</t>
+          <t>664299016</t>
         </is>
       </c>
       <c r="S71" s="3" t="inlineStr">
@@ -7308,7 +7316,7 @@
       </c>
       <c r="R90" s="3" t="inlineStr">
         <is>
-          <t>656566497</t>
+          <t>615748574</t>
         </is>
       </c>
       <c r="S90" s="3" t="inlineStr">
@@ -7397,7 +7405,7 @@
       </c>
       <c r="R91" s="3" t="inlineStr">
         <is>
-          <t>755638228</t>
+          <t>974310150</t>
         </is>
       </c>
       <c r="S91" s="3" t="inlineStr">
@@ -10677,8 +10685,16 @@
           <t xml:space="preserve">CLUB MUTANTE </t>
         </is>
       </c>
-      <c r="Q134" s="3" t="inlineStr"/>
-      <c r="R134" s="3" t="inlineStr"/>
+      <c r="Q134" s="3" t="inlineStr">
+        <is>
+          <t>ventanillaunica@borja.es</t>
+        </is>
+      </c>
+      <c r="R134" s="3" t="inlineStr">
+        <is>
+          <t>664054866</t>
+        </is>
+      </c>
       <c r="S134" s="3" t="inlineStr">
         <is>
           <t>https://borja.cumpletransparencia.es</t>
@@ -11438,7 +11454,7 @@
       <c r="Q144" s="3" t="inlineStr"/>
       <c r="R144" s="3" t="inlineStr">
         <is>
-          <t>753558549</t>
+          <t>791536509</t>
         </is>
       </c>
       <c r="S144" s="3" t="inlineStr">
@@ -11884,7 +11900,7 @@
       <c r="Q150" s="3" t="inlineStr"/>
       <c r="R150" s="3" t="inlineStr">
         <is>
-          <t>792324361</t>
+          <t>792317680</t>
         </is>
       </c>
       <c r="S150" s="3" t="inlineStr">
@@ -12088,8 +12104,16 @@
       <c r="N153" s="3" t="inlineStr"/>
       <c r="O153" s="3" t="inlineStr"/>
       <c r="P153" s="3" t="inlineStr"/>
-      <c r="Q153" s="3" t="inlineStr"/>
-      <c r="R153" s="3" t="inlineStr"/>
+      <c r="Q153" s="3" t="inlineStr">
+        <is>
+          <t>informacion@ayto-aviles.es</t>
+        </is>
+      </c>
+      <c r="R153" s="3" t="inlineStr">
+        <is>
+          <t>653394078</t>
+        </is>
+      </c>
       <c r="S153" s="3" t="inlineStr">
         <is>
           <t>https://aviles.es</t>
@@ -12164,7 +12188,7 @@
       </c>
       <c r="R154" s="3" t="inlineStr">
         <is>
-          <t>787239037</t>
+          <t>792310488</t>
         </is>
       </c>
       <c r="S154" s="3" t="inlineStr">
@@ -12335,8 +12359,16 @@
           <t>o explota, directa o indirectamente. Además, FOF recoge</t>
         </is>
       </c>
-      <c r="Q156" s="3" t="inlineStr"/>
-      <c r="R156" s="3" t="inlineStr"/>
+      <c r="Q156" s="3" t="inlineStr">
+        <is>
+          <t>ayuntamiento@viana.es</t>
+        </is>
+      </c>
+      <c r="R156" s="3" t="inlineStr">
+        <is>
+          <t>609110179</t>
+        </is>
+      </c>
       <c r="S156" s="3" t="inlineStr">
         <is>
           <t>http://www.viana.es</t>
@@ -13023,7 +13055,7 @@
       </c>
       <c r="R165" s="3" t="inlineStr">
         <is>
-          <t>722515367</t>
+          <t>600961018</t>
         </is>
       </c>
       <c r="S165" s="3" t="inlineStr">
@@ -13181,7 +13213,7 @@
       </c>
       <c r="R167" s="3" t="inlineStr">
         <is>
-          <t>623262727</t>
+          <t>626900413</t>
         </is>
       </c>
       <c r="S167" s="3" t="inlineStr">
@@ -14426,328 +14458,332 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Festa Presentació Vida Festival 2027: La Publicitat &amp; Bernal</t>
+          <t>Horteralia Cáceres 2026</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>Antiga Fàbrica Estrella Damm</t>
+          <t>Recinto Ferial de Cáceres</t>
         </is>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Cáceres</t>
         </is>
       </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="G185" s="3" t="inlineStr"/>
-      <c r="H185" s="2" t="inlineStr"/>
+          <t>Cáceres</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>Extremadura</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>Pop</t>
+        </is>
+      </c>
       <c r="I185" s="4" t="inlineStr">
         <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J185" s="2" t="inlineStr"/>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>CANO, CUPIDO, CYRIL KAMER</t>
+        </is>
+      </c>
       <c r="K185" s="2" t="inlineStr">
         <is>
-          <t>Vida Records &amp; Friends, Vida Festival</t>
-        </is>
-      </c>
-      <c r="L185" s="2" t="inlineStr"/>
+          <t>Camela, Ladilla rusa, Amatria, Cherri Coke, El Gato con Jotas, Los Desgraciaus, Los Inhumanos, Nebulossa, Sharonne</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mevoyacaceres.com/festival-horteralia-de-caceres/</t>
+        </is>
+      </c>
       <c r="M185" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N185" s="3" t="inlineStr"/>
+      <c r="N185" s="3" t="inlineStr">
+        <is>
+          <t>dpo@mediaprogramas.com</t>
+        </is>
+      </c>
       <c r="O185" s="3" t="inlineStr"/>
       <c r="P185" s="3" t="inlineStr">
         <is>
-          <t>Sitback Produccions, S.L.</t>
-        </is>
-      </c>
-      <c r="Q185" s="3" t="inlineStr"/>
-      <c r="R185" s="3" t="inlineStr"/>
-      <c r="S185" s="3" t="inlineStr"/>
+          <t>En Mediaprogramas S.L</t>
+        </is>
+      </c>
+      <c r="Q185" s="3" t="inlineStr">
+        <is>
+          <t>informacion@ayto-caceres.es</t>
+        </is>
+      </c>
+      <c r="R185" s="3" t="inlineStr">
+        <is>
+          <t>618380445</t>
+        </is>
+      </c>
+      <c r="S185" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ayto-caceres.es</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Horteralia Cáceres 2026</t>
+          <t>La CHICA FEST. Actuación de Elegante embustero. Formato trío</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>Recinto Ferial de Cáceres</t>
+          <t xml:space="preserve">Pub La chica de ayer </t>
         </is>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>Cáceres</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="F186" s="3" t="inlineStr">
         <is>
-          <t>Cáceres</t>
-        </is>
-      </c>
-      <c r="G186" s="3" t="inlineStr">
-        <is>
-          <t>Extremadura</t>
-        </is>
-      </c>
-      <c r="H186" s="2" t="inlineStr">
-        <is>
-          <t>Pop</t>
-        </is>
-      </c>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="G186" s="3" t="inlineStr"/>
+      <c r="H186" s="2" t="inlineStr"/>
       <c r="I186" s="4" t="inlineStr">
         <is>
-          <t>medio</t>
-        </is>
-      </c>
-      <c r="J186" s="2" t="inlineStr">
-        <is>
-          <t>CANO, CUPIDO, CYRIL KAMER</t>
-        </is>
-      </c>
-      <c r="K186" s="2" t="inlineStr">
-        <is>
-          <t>Camela, Ladilla rusa, Amatria, Cherri Coke, El Gato con Jotas, Los Desgraciaus, Los Inhumanos, Nebulossa, Sharonne</t>
-        </is>
-      </c>
-      <c r="L186" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mevoyacaceres.com/festival-horteralia-de-caceres/</t>
-        </is>
-      </c>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr"/>
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="2" t="inlineStr"/>
       <c r="M186" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N186" s="3" t="inlineStr">
-        <is>
-          <t>dpo@mediaprogramas.com</t>
-        </is>
-      </c>
+      <c r="N186" s="3" t="inlineStr"/>
       <c r="O186" s="3" t="inlineStr"/>
       <c r="P186" s="3" t="inlineStr">
         <is>
-          <t>En Mediaprogramas S.L</t>
-        </is>
-      </c>
-      <c r="Q186" s="3" t="inlineStr">
-        <is>
-          <t>informacion@ayto-caceres.es</t>
-        </is>
-      </c>
-      <c r="R186" s="3" t="inlineStr">
-        <is>
-          <t>618380445</t>
-        </is>
-      </c>
-      <c r="S186" s="3" t="inlineStr">
-        <is>
-          <t>https://www.ayto-caceres.es</t>
-        </is>
-      </c>
+          <t>La chica Fest</t>
+        </is>
+      </c>
+      <c r="Q186" s="3" t="inlineStr"/>
+      <c r="R186" s="3" t="inlineStr"/>
+      <c r="S186" s="3" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>La CHICA FEST. Actuación de Elegante embustero. Formato trío</t>
+          <t>Castañazo Rock 2026</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pub La chica de ayer </t>
+          <t>Mercado ganadero</t>
         </is>
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>Granada</t>
-        </is>
-      </c>
-      <c r="F187" s="3" t="inlineStr"/>
-      <c r="G187" s="3" t="inlineStr"/>
-      <c r="H187" s="2" t="inlineStr"/>
+          <t>Chantada</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>Lugo</t>
+        </is>
+      </c>
+      <c r="G187" s="3" t="inlineStr">
+        <is>
+          <t>Galicia</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>Urbano, Pop, Rock, Punk</t>
+        </is>
+      </c>
       <c r="I187" s="4" t="inlineStr">
         <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J187" s="2" t="inlineStr"/>
-      <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="2" t="inlineStr"/>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>CUPIDO, JUNNIO, CANO</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>Grande Amore, Kaotiko, Kumpania Algazarra, Moscow Death Brigade, Tremenda Jauría</t>
+        </is>
+      </c>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>https://castanhazo.com/venda-de-entradas/</t>
+        </is>
+      </c>
       <c r="M187" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N187" s="3" t="inlineStr"/>
+      <c r="N187" s="3" t="inlineStr">
+        <is>
+          <t>attcliente@woutick.es</t>
+        </is>
+      </c>
       <c r="O187" s="3" t="inlineStr"/>
-      <c r="P187" s="3" t="inlineStr">
-        <is>
-          <t>La chica Fest</t>
-        </is>
-      </c>
-      <c r="Q187" s="3" t="inlineStr"/>
-      <c r="R187" s="3" t="inlineStr"/>
-      <c r="S187" s="3" t="inlineStr"/>
+      <c r="P187" s="3" t="inlineStr"/>
+      <c r="Q187" s="3" t="inlineStr">
+        <is>
+          <t>concello@concellodechantada.es</t>
+        </is>
+      </c>
+      <c r="R187" s="3" t="inlineStr">
+        <is>
+          <t>614817558</t>
+        </is>
+      </c>
+      <c r="S187" s="3" t="inlineStr">
+        <is>
+          <t>https://www.concellodechantada.org</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Castañazo Rock 2026</t>
+          <t>GALILEO ROCK FEST</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>Mercado ganadero</t>
+          <t>Sala Galileo Galilei</t>
         </is>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>Chantada</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>Lugo</t>
-        </is>
-      </c>
-      <c r="G188" s="3" t="inlineStr">
-        <is>
-          <t>Galicia</t>
-        </is>
-      </c>
-      <c r="H188" s="2" t="inlineStr">
-        <is>
-          <t>Urbano, Pop, Rock, Punk</t>
-        </is>
-      </c>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr"/>
+      <c r="H188" s="2" t="inlineStr"/>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t>alto</t>
-        </is>
-      </c>
-      <c r="J188" s="2" t="inlineStr">
-        <is>
-          <t>CUPIDO, JUNNIO, CANO</t>
-        </is>
-      </c>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr"/>
       <c r="K188" s="2" t="inlineStr">
         <is>
-          <t>Grande Amore, Kaotiko, Kumpania Algazarra, Moscow Death Brigade, Tremenda Jauría</t>
-        </is>
-      </c>
-      <c r="L188" s="2" t="inlineStr">
-        <is>
-          <t>https://castanhazo.com/venda-de-entradas/</t>
-        </is>
-      </c>
+          <t>Lion Rock Fest</t>
+        </is>
+      </c>
+      <c r="L188" s="2" t="inlineStr"/>
       <c r="M188" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N188" s="3" t="inlineStr">
-        <is>
-          <t>attcliente@woutick.es</t>
-        </is>
-      </c>
+      <c r="N188" s="3" t="inlineStr"/>
       <c r="O188" s="3" t="inlineStr"/>
-      <c r="P188" s="3" t="inlineStr"/>
-      <c r="Q188" s="3" t="inlineStr">
-        <is>
-          <t>concello@concellodechantada.es</t>
-        </is>
-      </c>
-      <c r="R188" s="3" t="inlineStr">
-        <is>
-          <t>614817558</t>
-        </is>
-      </c>
-      <c r="S188" s="3" t="inlineStr">
-        <is>
-          <t>https://www.concellodechantada.org</t>
-        </is>
-      </c>
+      <c r="P188" s="3" t="inlineStr">
+        <is>
+          <t>Artisti-K Prod. Mus. y Cult, S.L.</t>
+        </is>
+      </c>
+      <c r="Q188" s="3" t="inlineStr"/>
+      <c r="R188" s="3" t="inlineStr"/>
+      <c r="S188" s="3" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>GALILEO ROCK FEST</t>
+          <t>ALFAJARÍN, CULTURA ELECTRÓNICA 2026 (The Raven Clan)</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>Sala Galileo Galilei</t>
+          <t xml:space="preserve">SALÓN CULTURAL “LA PORTAZA” </t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Alfajarín</t>
         </is>
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Alfajarín</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr"/>
@@ -14758,11 +14794,7 @@
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr"/>
-      <c r="K189" s="2" t="inlineStr">
-        <is>
-          <t>Lion Rock Fest</t>
-        </is>
-      </c>
+      <c r="K189" s="2" t="inlineStr"/>
       <c r="L189" s="2" t="inlineStr"/>
       <c r="M189" s="2" t="inlineStr">
         <is>
@@ -14773,7 +14805,7 @@
       <c r="O189" s="3" t="inlineStr"/>
       <c r="P189" s="3" t="inlineStr">
         <is>
-          <t>Artisti-K Prod. Mus. y Cult, S.L.</t>
+          <t>AYUNTAMIENTO DE ALFAJARÍN</t>
         </is>
       </c>
       <c r="Q189" s="3" t="inlineStr"/>
@@ -14783,7 +14815,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>ALFAJARÍN, CULTURA ELECTRÓNICA 2026 (The Raven Clan)</t>
+          <t>IV FESTIVAL SEVILLA SIXTIES SOUND</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -14798,15 +14830,19 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SALÓN CULTURAL “LA PORTAZA” </t>
+          <t>SALA EVEN</t>
         </is>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>Alfajarín</t>
-        </is>
-      </c>
-      <c r="F190" s="3" t="inlineStr"/>
+          <t>SEVILLA</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="inlineStr">
+        <is>
+          <t>SEVILLA</t>
+        </is>
+      </c>
       <c r="G190" s="3" t="inlineStr"/>
       <c r="H190" s="2" t="inlineStr"/>
       <c r="I190" s="4" t="inlineStr">
@@ -14826,7 +14862,7 @@
       <c r="O190" s="3" t="inlineStr"/>
       <c r="P190" s="3" t="inlineStr">
         <is>
-          <t>AYUNTAMIENTO DE ALFAJARÍN</t>
+          <t>SIXTIES SOUND SEVILLA</t>
         </is>
       </c>
       <c r="Q190" s="3" t="inlineStr"/>
@@ -14836,30 +14872,34 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>IV FESTIVAL SEVILLA SIXTIES SOUND</t>
+          <t>IBERDROLA MUSIC FESTIVAL VALENCIA - CONCIERTO ESTOPA</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>2026-11-21</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>2026-11-21</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>SALA EVEN</t>
+          <t>Roig Arena</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>SEVILLA</t>
-        </is>
-      </c>
-      <c r="F191" s="3" t="inlineStr"/>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
       <c r="G191" s="3" t="inlineStr"/>
       <c r="H191" s="2" t="inlineStr"/>
       <c r="I191" s="4" t="inlineStr">
@@ -14868,7 +14908,11 @@
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr"/>
-      <c r="K191" s="2" t="inlineStr"/>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>IBERDROLA MUSIC FESTIVAL VALENCIA, Estopa</t>
+        </is>
+      </c>
       <c r="L191" s="2" t="inlineStr"/>
       <c r="M191" s="2" t="inlineStr">
         <is>
@@ -14879,7 +14923,7 @@
       <c r="O191" s="3" t="inlineStr"/>
       <c r="P191" s="3" t="inlineStr">
         <is>
-          <t>SIXTIES SOUND SEVILLA</t>
+          <t>Live Nation España S.A.U.</t>
         </is>
       </c>
       <c r="Q191" s="3" t="inlineStr"/>
@@ -14889,7 +14933,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>IBERDROLA MUSIC FESTIVAL VALENCIA - CONCIERTO ESTOPA</t>
+          <t>Metal Bee 2026</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -14904,21 +14948,29 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>Roig Arena</t>
+          <t>Sala Matadero</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
+          <t>Ayora</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
           <t>Valencia</t>
         </is>
       </c>
-      <c r="F192" s="3" t="inlineStr">
-        <is>
-          <t>Valencia</t>
-        </is>
-      </c>
-      <c r="G192" s="3" t="inlineStr"/>
-      <c r="H192" s="2" t="inlineStr"/>
+      <c r="G192" s="3" t="inlineStr">
+        <is>
+          <t>Comunidad Valenciana</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>Metal</t>
+        </is>
+      </c>
       <c r="I192" s="4" t="inlineStr">
         <is>
           <t>bajo</t>
@@ -14927,146 +14979,142 @@
       <c r="J192" s="2" t="inlineStr"/>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>IBERDROLA MUSIC FESTIVAL VALENCIA, Estopa</t>
-        </is>
-      </c>
-      <c r="L192" s="2" t="inlineStr"/>
+          <t>Leo Jiménez, Débler Eternia, Salduie, Seventh Hell, Six Burning Knives</t>
+        </is>
+      </c>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>http://tickets.salamatadero.com/es/matadero-live-music/iv-festival-metalbee/2026-11-28/</t>
+        </is>
+      </c>
       <c r="M192" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N192" s="3" t="inlineStr"/>
+      <c r="N192" s="3" t="inlineStr">
+        <is>
+          <t>salamatadero@gmail.com</t>
+        </is>
+      </c>
       <c r="O192" s="3" t="inlineStr"/>
-      <c r="P192" s="3" t="inlineStr">
-        <is>
-          <t>Live Nation España S.A.U.</t>
-        </is>
-      </c>
+      <c r="P192" s="3" t="inlineStr"/>
       <c r="Q192" s="3" t="inlineStr"/>
       <c r="R192" s="3" t="inlineStr"/>
-      <c r="S192" s="3" t="inlineStr"/>
+      <c r="S192" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ayora.es</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Metal Bee 2026</t>
+          <t>NoTeMofest acto 4</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2027-02-20</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2027-02-20</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>Sala Matadero</t>
+          <t>Andén 56</t>
         </is>
       </c>
       <c r="E193" s="3" t="inlineStr">
         <is>
-          <t>Ayora</t>
+          <t>Burgos</t>
         </is>
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>Valencia</t>
-        </is>
-      </c>
-      <c r="G193" s="3" t="inlineStr">
-        <is>
-          <t>Comunidad Valenciana</t>
-        </is>
-      </c>
-      <c r="H193" s="2" t="inlineStr">
-        <is>
-          <t>Metal</t>
-        </is>
-      </c>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="G193" s="3" t="inlineStr"/>
+      <c r="H193" s="2" t="inlineStr"/>
       <c r="I193" s="4" t="inlineStr">
         <is>
           <t>bajo</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr"/>
-      <c r="K193" s="2" t="inlineStr">
-        <is>
-          <t>Leo Jiménez, Débler Eternia, Salduie, Seventh Hell, Six Burning Knives</t>
-        </is>
-      </c>
-      <c r="L193" s="2" t="inlineStr">
-        <is>
-          <t>http://tickets.salamatadero.com/es/matadero-live-music/iv-festival-metalbee/2026-11-28/</t>
-        </is>
-      </c>
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="2" t="inlineStr"/>
       <c r="M193" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N193" s="3" t="inlineStr">
-        <is>
-          <t>salamatadero@gmail.com</t>
-        </is>
-      </c>
+      <c r="N193" s="3" t="inlineStr"/>
       <c r="O193" s="3" t="inlineStr"/>
-      <c r="P193" s="3" t="inlineStr"/>
-      <c r="Q193" s="3" t="inlineStr">
-        <is>
-          <t>registro@ayora.es</t>
-        </is>
-      </c>
-      <c r="R193" s="3" t="inlineStr">
-        <is>
-          <t>880898509</t>
-        </is>
-      </c>
-      <c r="S193" s="3" t="inlineStr">
-        <is>
-          <t>https://www.ayora.es</t>
-        </is>
-      </c>
+      <c r="P193" s="3" t="inlineStr">
+        <is>
+          <t>Steel Souls Producciones</t>
+        </is>
+      </c>
+      <c r="Q193" s="3" t="inlineStr"/>
+      <c r="R193" s="3" t="inlineStr"/>
+      <c r="S193" s="3" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>NoTeMofest acto 4</t>
+          <t>Viña Rock 2027</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>2027-02-20</t>
+          <t>2027-04-29</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>2027-02-20</t>
+          <t>2027-05-01</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>Andén 56</t>
+          <t>Recinto Ferial de Villarrobledo</t>
         </is>
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>Burgos</t>
-        </is>
-      </c>
-      <c r="F194" s="3" t="inlineStr"/>
-      <c r="G194" s="3" t="inlineStr"/>
-      <c r="H194" s="2" t="inlineStr"/>
+          <t>Villarrobledo</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="G194" s="3" t="inlineStr">
+        <is>
+          <t>Castilla-La Mancha</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>Rock</t>
+        </is>
+      </c>
       <c r="I194" s="4" t="inlineStr">
         <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J194" s="2" t="inlineStr"/>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>CUPIDO, JUNNIO</t>
+        </is>
+      </c>
       <c r="K194" s="2" t="inlineStr"/>
       <c r="L194" s="2" t="inlineStr"/>
       <c r="M194" s="2" t="inlineStr">
@@ -15076,122 +15124,122 @@
       </c>
       <c r="N194" s="3" t="inlineStr"/>
       <c r="O194" s="3" t="inlineStr"/>
-      <c r="P194" s="3" t="inlineStr">
-        <is>
-          <t>Steel Souls Producciones</t>
-        </is>
-      </c>
+      <c r="P194" s="3" t="inlineStr"/>
       <c r="Q194" s="3" t="inlineStr"/>
-      <c r="R194" s="3" t="inlineStr"/>
-      <c r="S194" s="3" t="inlineStr"/>
+      <c r="R194" s="3" t="inlineStr">
+        <is>
+          <t>736908127</t>
+        </is>
+      </c>
+      <c r="S194" s="3" t="inlineStr">
+        <is>
+          <t>https://villarrobledo.com</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Viña Rock 2027</t>
+          <t>Interestelar Sevilla 2027</t>
         </is>
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>2027-04-29</t>
+          <t>2027-05-14</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-05-15</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Recinto Ferial de Villarrobledo</t>
+          <t>Centro Andaluz de Arte Contemporáneo</t>
         </is>
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
-          <t>Villarrobledo</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>Albacete</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="G195" s="3" t="inlineStr">
         <is>
-          <t>Castilla-La Mancha</t>
-        </is>
-      </c>
-      <c r="H195" s="2" t="inlineStr">
-        <is>
-          <t>Rock</t>
-        </is>
-      </c>
+          <t>Andalucía</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr"/>
       <c r="I195" s="4" t="inlineStr">
         <is>
-          <t>medio</t>
-        </is>
-      </c>
-      <c r="J195" s="2" t="inlineStr">
-        <is>
-          <t>CUPIDO, JUNNIO</t>
-        </is>
-      </c>
+          <t>bajo</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr"/>
       <c r="K195" s="2" t="inlineStr"/>
-      <c r="L195" s="2" t="inlineStr"/>
+      <c r="L195" s="2" t="inlineStr">
+        <is>
+          <t>https://conciertosensevilla.es/interestelar-sevilla-2027-viva-suecia-y-la-oreja-de-van-gogh-primeros-nombres-del-cartel/</t>
+        </is>
+      </c>
       <c r="M195" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N195" s="3" t="inlineStr"/>
+      <c r="N195" s="3" t="inlineStr">
+        <is>
+          <t>hola@conciertosensevilla.es</t>
+        </is>
+      </c>
       <c r="O195" s="3" t="inlineStr"/>
       <c r="P195" s="3" t="inlineStr"/>
       <c r="Q195" s="3" t="inlineStr"/>
-      <c r="R195" s="3" t="inlineStr">
-        <is>
-          <t>736908127</t>
-        </is>
-      </c>
+      <c r="R195" s="3" t="inlineStr"/>
       <c r="S195" s="3" t="inlineStr">
         <is>
-          <t>https://villarrobledo.com</t>
+          <t>https://www.discoversevilla.city</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Interestelar Sevilla 2027</t>
+          <t>Primavera Sound Barcelona 2027</t>
         </is>
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>2027-05-14</t>
+          <t>2027-06-03</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>2027-05-15</t>
+          <t>2027-06-05</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>Centro Andaluz de Arte Contemporáneo</t>
+          <t>Parc del Fòrum</t>
         </is>
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="F196" s="3" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="G196" s="3" t="inlineStr">
         <is>
-          <t>Andalucía</t>
+          <t>Cataluña</t>
         </is>
       </c>
       <c r="H196" s="2" t="inlineStr"/>
@@ -15202,50 +15250,46 @@
       </c>
       <c r="J196" s="2" t="inlineStr"/>
       <c r="K196" s="2" t="inlineStr"/>
-      <c r="L196" s="2" t="inlineStr">
-        <is>
-          <t>https://conciertosensevilla.es/interestelar-sevilla-2027-viva-suecia-y-la-oreja-de-van-gogh-primeros-nombres-del-cartel/</t>
-        </is>
-      </c>
+      <c r="L196" s="2" t="inlineStr"/>
       <c r="M196" s="2" t="inlineStr">
         <is>
           <t>confirmado</t>
         </is>
       </c>
-      <c r="N196" s="3" t="inlineStr">
-        <is>
-          <t>hola@conciertosensevilla.es</t>
-        </is>
-      </c>
+      <c r="N196" s="3" t="inlineStr"/>
       <c r="O196" s="3" t="inlineStr"/>
       <c r="P196" s="3" t="inlineStr"/>
       <c r="Q196" s="3" t="inlineStr"/>
-      <c r="R196" s="3" t="inlineStr"/>
+      <c r="R196" s="3" t="inlineStr">
+        <is>
+          <t>616401389</t>
+        </is>
+      </c>
       <c r="S196" s="3" t="inlineStr">
         <is>
-          <t>https://www.discoversevilla.city</t>
+          <t>https://ajuntament.barcelona.cat</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Primavera Sound Barcelona 2027</t>
+          <t>Sónar 2027</t>
         </is>
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>2027-06-03</t>
+          <t>2027-06-17</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>2027-06-05</t>
+          <t>2027-06-19</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>Parc del Fòrum</t>
+          <t>Sónar de día - Fira Montjuïc</t>
         </is>
       </c>
       <c r="E197" s="3" t="inlineStr">
@@ -15295,39 +15339,35 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Sónar 2027</t>
+          <t>Scanner bilbao</t>
         </is>
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>2027-06-17</t>
+          <t>2027-09-17</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>2027-06-19</t>
+          <t>2027-09-17</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Sónar de día - Fira Montjuïc</t>
+          <t>D8 sorkuntza</t>
         </is>
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Bilbao</t>
         </is>
       </c>
       <c r="F198" s="3" t="inlineStr">
         <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="G198" s="3" t="inlineStr">
-        <is>
-          <t>Cataluña</t>
-        </is>
-      </c>
+          <t>Bilbao</t>
+        </is>
+      </c>
+      <c r="G198" s="3" t="inlineStr"/>
       <c r="H198" s="2" t="inlineStr"/>
       <c r="I198" s="4" t="inlineStr">
         <is>
@@ -15344,135 +15384,17 @@
       </c>
       <c r="N198" s="3" t="inlineStr"/>
       <c r="O198" s="3" t="inlineStr"/>
-      <c r="P198" s="3" t="inlineStr"/>
+      <c r="P198" s="3" t="inlineStr">
+        <is>
+          <t>Copilots Events</t>
+        </is>
+      </c>
       <c r="Q198" s="3" t="inlineStr"/>
-      <c r="R198" s="3" t="inlineStr">
-        <is>
-          <t>616401389</t>
-        </is>
-      </c>
-      <c r="S198" s="3" t="inlineStr">
-        <is>
-          <t>https://ajuntament.barcelona.cat</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="2" t="inlineStr">
-        <is>
-          <t>All Access Pass + Bus Super Early Bird - Circuit Festival 2027</t>
-        </is>
-      </c>
-      <c r="B199" s="3" t="inlineStr">
-        <is>
-          <t>2027-08-15</t>
-        </is>
-      </c>
-      <c r="C199" s="3" t="inlineStr">
-        <is>
-          <t>2027-08-15</t>
-        </is>
-      </c>
-      <c r="D199" s="2" t="inlineStr">
-        <is>
-          <t>Varios Recintos</t>
-        </is>
-      </c>
-      <c r="E199" s="3" t="inlineStr">
-        <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="F199" s="3" t="inlineStr">
-        <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="G199" s="3" t="inlineStr"/>
-      <c r="H199" s="2" t="inlineStr"/>
-      <c r="I199" s="4" t="inlineStr">
-        <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J199" s="2" t="inlineStr"/>
-      <c r="K199" s="2" t="inlineStr">
-        <is>
-          <t>Circuit Festival</t>
-        </is>
-      </c>
-      <c r="L199" s="2" t="inlineStr"/>
-      <c r="M199" s="2" t="inlineStr">
-        <is>
-          <t>confirmado</t>
-        </is>
-      </c>
-      <c r="N199" s="3" t="inlineStr"/>
-      <c r="O199" s="3" t="inlineStr"/>
-      <c r="P199" s="3" t="inlineStr">
-        <is>
-          <t>Matinée 2000, SLU</t>
-        </is>
-      </c>
-      <c r="Q199" s="3" t="inlineStr"/>
-      <c r="R199" s="3" t="inlineStr"/>
-      <c r="S199" s="3" t="inlineStr"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
-        <is>
-          <t>Scanner bilbao</t>
-        </is>
-      </c>
-      <c r="B200" s="3" t="inlineStr">
-        <is>
-          <t>2027-09-17</t>
-        </is>
-      </c>
-      <c r="C200" s="3" t="inlineStr">
-        <is>
-          <t>2027-09-17</t>
-        </is>
-      </c>
-      <c r="D200" s="2" t="inlineStr">
-        <is>
-          <t>D8 sorkuntza</t>
-        </is>
-      </c>
-      <c r="E200" s="3" t="inlineStr">
-        <is>
-          <t>Bilbao</t>
-        </is>
-      </c>
-      <c r="F200" s="3" t="inlineStr"/>
-      <c r="G200" s="3" t="inlineStr"/>
-      <c r="H200" s="2" t="inlineStr"/>
-      <c r="I200" s="4" t="inlineStr">
-        <is>
-          <t>bajo</t>
-        </is>
-      </c>
-      <c r="J200" s="2" t="inlineStr"/>
-      <c r="K200" s="2" t="inlineStr"/>
-      <c r="L200" s="2" t="inlineStr"/>
-      <c r="M200" s="2" t="inlineStr">
-        <is>
-          <t>confirmado</t>
-        </is>
-      </c>
-      <c r="N200" s="3" t="inlineStr"/>
-      <c r="O200" s="3" t="inlineStr"/>
-      <c r="P200" s="3" t="inlineStr">
-        <is>
-          <t>Copilots Events</t>
-        </is>
-      </c>
-      <c r="Q200" s="3" t="inlineStr"/>
-      <c r="R200" s="3" t="inlineStr"/>
-      <c r="S200" s="3" t="inlineStr"/>
+      <c r="R198" s="3" t="inlineStr"/>
+      <c r="S198" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S200"/>
+  <autoFilter ref="A1:S198"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15505,7 +15427,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>18/10/2026 09:54</t>
+          <t>18/10/2026 13:47</t>
         </is>
       </c>
     </row>
@@ -15516,7 +15438,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4">
@@ -15526,7 +15448,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -15613,7 +15535,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15">
@@ -15633,7 +15555,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">

</xml_diff>